<commit_message>
Rapor modülü (kapak, üst/alt bilgi, içindekiler), harmonik/yan-band imleçleri, WAV içe aktarma, bit akışı (12/14 bit) alanları, şablon güncellemesi
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014rd2szXiJ1bnHEWArCLqeb
</commit_message>
<xml_diff>
--- a/sablon/MATView_Cerceve_Sablonu.xlsx
+++ b/sablon/MATView_Cerceve_Sablonu.xlsx
@@ -63897,7 +63897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -64507,17 +64507,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ADC_KANAL</t>
+          <t>PAKET12_A</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SENSOR_1</t>
+          <t>SENSOR_101</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>u16</t>
+          <t>ub</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -64525,17 +64525,13 @@
           <t>BE</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>(x-2048)/4096*5</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>1</v>
       </c>
@@ -64543,6 +64539,90 @@
         <v>0</v>
       </c>
       <c r="J15" t="inlineStr">
+        <is>
+          <t>12 bit paketli (bit akışı): 1. örnek, bitler 0-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PAKET12_B</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SENSOR_101</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ub</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>12-23</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>12 bit paketli: 2. örnek (aynı 3 baytta), bitler 12-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ADC_KANAL</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SENSOR_1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>u16</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>(x-2048)/4096*5</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>12 bit ADC sayısını 0–5 V’a çevirme (örnek)</t>
         </is>
@@ -64567,7 +64647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -64699,26 +64779,43 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>ub / sb</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Bit akışı (işaretsiz/işaretli): Bit = a-b, başlangıç baytının en anlamlı bitinden sayılır (0=ilk bit), en çok 32 bit; 12/14 bit paketli telemetre için</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>f64</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>IEEE-754 çift duyarlık</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Formül işlevleri</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr">
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
         <is>
           <t>x, + − * / ^, ( ), abs sqrt sin cos tan exp log log10 sign round floor ceil atan2(a,b) pow(a,b) max(a,b) min(a,b) ve başka alan adları</t>
         </is>

</xml_diff>